<commit_message>
Planners: precios del catalogo, siempre terminados en 990
- Precios del catalogo de planners (Canva) llevados a 990: $11.990 los de
  100 hojas (Universitario, Mi Planner, Diario, Brilla, Semanal Diario,
  Control de Gastos, Docente, Gratitud, Suena en Grande), $7.990 Semanal,
  Diario anillado arriba y Recetas, $9.990 100 Citas Juntos.
- Regla a990: todo precio (planilla o con descuento) se muestra terminado en
  990; el tachado del descuento tambien.
- Detalles con las hojas del catalogo: 100 o 70 hojas de 106 g, anillado
  metalico blanco.
- Plantilla de la planilla con los mismos precios y la regla en leeme.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planners_heart_graphic.xlsx
+++ b/planners_heart_graphic.xlsx
@@ -147,7 +147,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Número sin signo ni puntos (24990). Vacío = 'Consultar' y sin carrito.</t>
+          <t xml:space="preserve">Número sin signo ni puntos (11990). Vacío = 'Consultar' y sin carrito. La web siempre lo muestra terminado en 990: si escribes 12000 se ve $11.990 (también con descuento).</t>
         </is>
       </c>
     </row>
@@ -499,6 +499,9 @@
           <t xml:space="preserve">Mi Planner</t>
         </is>
       </c>
+      <c r="D3" s="0">
+        <v>11990</v>
+      </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -511,7 +514,7 @@
       </c>
       <c r="H3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K3" s="0" t="inlineStr">
@@ -541,6 +544,9 @@
           <t xml:space="preserve">Planner Brilla</t>
         </is>
       </c>
+      <c r="D4" s="0">
+        <v>11990</v>
+      </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -553,7 +559,7 @@
       </c>
       <c r="H4" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
@@ -583,6 +589,9 @@
           <t xml:space="preserve">Planner Docente · Héroes</t>
         </is>
       </c>
+      <c r="D5" s="0">
+        <v>11990</v>
+      </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -595,7 +604,7 @@
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
@@ -625,6 +634,9 @@
           <t xml:space="preserve">Planner Docente</t>
         </is>
       </c>
+      <c r="D6" s="0">
+        <v>11990</v>
+      </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -637,7 +649,7 @@
       </c>
       <c r="H6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K6" s="0" t="inlineStr">
@@ -667,6 +679,9 @@
           <t xml:space="preserve">Planner Universitario</t>
         </is>
       </c>
+      <c r="D7" s="0">
+        <v>11990</v>
+      </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -679,7 +694,7 @@
       </c>
       <c r="H7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K7" s="0" t="inlineStr">
@@ -709,6 +724,9 @@
           <t xml:space="preserve">Planner Diario</t>
         </is>
       </c>
+      <c r="D8" s="0">
+        <v>11990</v>
+      </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -721,7 +739,7 @@
       </c>
       <c r="H8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K8" s="0" t="inlineStr">
@@ -751,6 +769,9 @@
           <t xml:space="preserve">Planner Diario · Anillado arriba</t>
         </is>
       </c>
+      <c r="D9" s="0">
+        <v>7990</v>
+      </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -763,7 +784,7 @@
       </c>
       <c r="H9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K9" s="0" t="inlineStr">
@@ -793,6 +814,9 @@
           <t xml:space="preserve">Planner Semanal Diario</t>
         </is>
       </c>
+      <c r="D10" s="0">
+        <v>11990</v>
+      </c>
       <c r="F10" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -805,7 +829,7 @@
       </c>
       <c r="H10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K10" s="0" t="inlineStr">
@@ -835,6 +859,9 @@
           <t xml:space="preserve">Planner Sueña en Grande</t>
         </is>
       </c>
+      <c r="D11" s="0">
+        <v>11990</v>
+      </c>
       <c r="F11" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -847,7 +874,7 @@
       </c>
       <c r="H11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K11" s="0" t="inlineStr">
@@ -877,6 +904,9 @@
           <t xml:space="preserve">Diario de Gratitud</t>
         </is>
       </c>
+      <c r="D12" s="0">
+        <v>11990</v>
+      </c>
       <c r="F12" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -889,7 +919,7 @@
       </c>
       <c r="H12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K12" s="0" t="inlineStr">
@@ -919,6 +949,9 @@
           <t xml:space="preserve">Planner Control de Gastos</t>
         </is>
       </c>
+      <c r="D13" s="0">
+        <v>11990</v>
+      </c>
       <c r="F13" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -931,7 +964,7 @@
       </c>
       <c r="H13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K13" s="0" t="inlineStr">
@@ -961,6 +994,9 @@
           <t xml:space="preserve">100 Citas Juntos</t>
         </is>
       </c>
+      <c r="D14" s="0">
+        <v>9990</v>
+      </c>
       <c r="F14" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -973,7 +1009,7 @@
       </c>
       <c r="H14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K14" s="0" t="inlineStr">
@@ -1129,6 +1165,9 @@
           <t xml:space="preserve">Agenda Mis Recetas</t>
         </is>
       </c>
+      <c r="D18" s="0">
+        <v>7990</v>
+      </c>
       <c r="F18" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -1141,7 +1180,7 @@
       </c>
       <c r="H18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K18" s="0" t="inlineStr">
@@ -1172,7 +1211,7 @@
         </is>
       </c>
       <c r="D19" s="0">
-        <v>9990</v>
+        <v>7990</v>
       </c>
       <c r="F19" s="0" t="inlineStr">
         <is>
@@ -1186,7 +1225,7 @@
       </c>
       <c r="H19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tamaño A5 apaisado (21 × 14,8 cm) · anillado</t>
+          <t xml:space="preserve">TamaÃ±o A5 apaisado (21 Ã 14,8 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
       </c>
       <c r="K19" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Planners: precios del resto (A6, Carnet, 100 Citas, Docente Heroes)
- A6 (Mini Planner Diario, Mini Agenda Lineas, Mini Planner Semanal, Mis
  Pedidos): $5.990; Mini Planner de Escritorio: $6.990.
- Carnet de Control Veterinario, 100 Citas con Amigas y con Mama: $9.990.
- Planner Docente Heroes: $9.990 (el otro Docente sigue en $11.990).
- Ya no queda ningun planner en Consultar. Plantilla actualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planners_heart_graphic.xlsx
+++ b/planners_heart_graphic.xlsx
@@ -590,7 +590,7 @@
         </is>
       </c>
       <c r="D5" s="0">
-        <v>11990</v>
+        <v>9990</v>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
@@ -604,7 +604,7 @@
       </c>
       <c r="H5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
+          <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· anillado</t>
         </is>
       </c>
       <c r="K5" s="0" t="inlineStr">
@@ -1039,6 +1039,9 @@
           <t xml:space="preserve">100 Citas con Amigas</t>
         </is>
       </c>
+      <c r="D15" s="0">
+        <v>9990</v>
+      </c>
       <c r="F15" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -1081,6 +1084,9 @@
           <t xml:space="preserve">100 Citas con Mamá</t>
         </is>
       </c>
+      <c r="D16" s="0">
+        <v>9990</v>
+      </c>
       <c r="F16" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -1123,6 +1129,9 @@
           <t xml:space="preserve">Carnet de Control Veterinario</t>
         </is>
       </c>
+      <c r="D17" s="0">
+        <v>9990</v>
+      </c>
       <c r="F17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
@@ -1255,6 +1264,9 @@
           <t xml:space="preserve">Mini Planner Diario</t>
         </is>
       </c>
+      <c r="D20" s="0">
+        <v>5990</v>
+      </c>
       <c r="F20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A6</t>
@@ -1297,6 +1309,9 @@
           <t xml:space="preserve">Mini Agenda Líneas</t>
         </is>
       </c>
+      <c r="D21" s="0">
+        <v>5990</v>
+      </c>
       <c r="F21" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A6</t>
@@ -1339,6 +1354,9 @@
           <t xml:space="preserve">Mini Planner Semanal</t>
         </is>
       </c>
+      <c r="D22" s="0">
+        <v>5990</v>
+      </c>
       <c r="F22" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A6</t>
@@ -1381,6 +1399,9 @@
           <t xml:space="preserve">Agenda Mis Pedidos</t>
         </is>
       </c>
+      <c r="D23" s="0">
+        <v>5990</v>
+      </c>
       <c r="F23" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">A6</t>
@@ -1422,6 +1443,9 @@
         <is>
           <t xml:space="preserve">Mini Planner de Escritorio</t>
         </is>
+      </c>
+      <c r="D24" s="0">
+        <v>6990</v>
       </c>
       <c r="F24" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Planners: Atrevete B5 a $14.990 y orden por tamano y precio
El catalogo va de mayor a menor tamano (B5, A5, A6) y, dentro de cada
tamano, del precio mas alto al mas bajo; la columna orden de la planilla
solo desempata a igual tamano y precio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planners_heart_graphic.xlsx
+++ b/planners_heart_graphic.xlsx
@@ -207,7 +207,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opcional. Número para ordenar dentro de cada tamaño (1 primero).</t>
+          <t xml:space="preserve">La web ordena por tamaño (B5, A5, A6) y, dentro de cada tamaño, del precio más alto al más bajo. orden es opcional: decide entre planners del mismo tamaño y precio (1 primero).</t>
         </is>
       </c>
     </row>
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="D2" s="0">
-        <v>24990</v>
+        <v>14990</v>
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Planners: dentro de cada tamano, planners primero y agendas tematicas al final
Orden: tamano (B5, A5, A6) > planners antes que agendas de otra tematica
(tema: true: Gratitud, 100 Citas, Carnet, Recetas, Mis Pedidos, Mini Agenda
Lineas) > precio de mayor a menor > orden de la planilla. La planilla suma la
columna tipo (planner / tematica).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planners_heart_graphic.xlsx
+++ b/planners_heart_graphic.xlsx
@@ -207,149 +207,161 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La web ordena por tamaño (B5, A5, A6) y, dentro de cada tamaño, del precio más alto al más bajo. orden es opcional: decide entre planners del mismo tamaño y precio (1 primero).</t>
+          <t xml:space="preserve">La web ordena por tamaño (B5, A5, A6); dentro de cada tamaño van primero los planners y al final las agendas de otra temática, cada grupo del precio más alto al más bajo. orden es opcional: decide entre los del mismo tamaño, tipo y precio (1 primero).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners · anillado / orientacion</t>
+          <t xml:space="preserve">planners · tipo</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">anillado: costado o arriba. orientacion: vertical o apaisada. Solo hace falta para planners nuevos.</t>
+          <t xml:space="preserve">planner (planificación: semanal, diaria, mensual, docente…) o tematica (agendas de otra temática: 100 Citas, recetas, carnet veterinario, gratitud, pedidos…). Las temáticas van al final de su tamaño.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners · fila config</t>
+          <t xml:space="preserve">planners · anillado / orientacion</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La fila con id = config guarda en precio el valor de 'Personaliza tu portada' (hoy 1000).</t>
+          <t xml:space="preserve">anillado: costado o arriba. orientacion: vertical o apaisada. Solo hace falta para planners nuevos.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Planner nuevo</t>
+          <t xml:space="preserve">planners · fila config</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agrega una fila en planners con un id nuevo (sin espacios, ej. agenda-flores) y al menos una portada en planners_portadas con ese mismo id. Sus hojas van en planners_hojas.</t>
+          <t xml:space="preserve">La fila con id = config guarda en precio el valor de 'Personaliza tu portada' (hoy 1000).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners_portadas</t>
+          <t xml:space="preserve">Planner nuevo</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una fila por portada NUEVA (se suma a las que ya existen). id_planner, orden (posición entre las nuevas), nombre (se ve en la web), url_portada (obligatoria), url_contratapa (opcional; vacío = contratapa lisa), color (opcional, ej. #ffc7e5, para la contratapa lisa), activo (si / no).</t>
+          <t xml:space="preserve">Agrega una fila en planners con un id nuevo (sin espacios, ej. agenda-flores) y al menos una portada en planners_portadas con ese mismo id. Sus hojas van en planners_hojas.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners_portadas · interior</t>
+          <t xml:space="preserve">planners_portadas</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una portada nueva muestra el interior de la primera portada del planner, más las hojas de planners_hojas que tengan su número en la columna portada.</t>
+          <t xml:space="preserve">Una fila por portada NUEVA (se suma a las que ya existen). id_planner, orden (posición entre las nuevas), nombre (se ve en la web), url_portada (obligatoria), url_contratapa (opcional; vacío = contratapa lisa), color (opcional, ej. #ffc7e5, para la contratapa lisa), activo (si / no).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners_hojas</t>
+          <t xml:space="preserve">planners_portadas · interior</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una fila por hoja que se SUMA al final del interior (antes de la contratapa). id_planner, portada (vacío = todas; o el número de portada como se ve en la web), orden, titulo (se ve bajo el visor), url, pliego, repetir.</t>
+          <t xml:space="preserve">Una portada nueva muestra el interior de la primera portada del planner, más las hojas de planners_hojas que tengan su número en la columna portada.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners_hojas · url</t>
+          <t xml:space="preserve">planners_hojas</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Una imagen en internet (https://…, idealmente Cloudinary) o el archivo de una hoja que el planner YA tiene (ej. pagina-1-03.jpg): búscalo en la pestaña hojas_actuales.</t>
+          <t xml:space="preserve">Una fila por hoja que se SUMA al final del interior (antes de la contratapa). id_planner, portada (vacío = todas; o el número de portada como se ve en la web), orden, titulo (se ve bajo el visor), url, pliego, repetir.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners_hojas · repetir</t>
+          <t xml:space="preserve">planners_hojas · url</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cuántas veces se repite esa hoja (ej. 5). Sirve para mostrar varias hojas de cuadros, líneas, notas o recetas. Máximo 50.</t>
+          <t xml:space="preserve">Una imagen en internet (https://…, idealmente Cloudinary) o el archivo de una hoja que el planner YA tiene (ej. pagina-1-03.jpg): búscalo en la pestaña hojas_actuales.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">planners_hojas · pliego</t>
+          <t xml:space="preserve">planners_hojas · repetir</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">si = esa hoja y la siguiente se ven juntas, abiertas como pliego (izquierda + derecha). Con repetir, se repite el pliego completo.</t>
+          <t xml:space="preserve">Cuántas veces se repite esa hoja (ej. 5). Sirve para mostrar varias hojas de cuadros, líneas, notas o recetas. Máximo 50.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ejemplo: repetir cuadros</t>
+          <t xml:space="preserve">planners_hojas · pliego</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Para que el Sueña en Grande Azul tenga 6 hojas de cuadros más: en planners_hojas → id_planner: suena · portada: 1 · titulo: Notas · url: pagina-1-03.jpg · repetir: 6.</t>
+          <t xml:space="preserve">si = esa hoja y la siguiente se ven juntas, abiertas como pliego (izquierda + derecha). Con repetir, se repite el pliego completo.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">hojas_actuales</t>
+          <t xml:space="preserve">Ejemplo: repetir cuadros</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Solo referencia (la web no la lee): cada hoja que hoy tiene cada planner, con su título y su archivo. portada 'todas' = la misma hoja en todas las portadas.</t>
+          <t xml:space="preserve">Para que el Sueña en Grande Azul tenga 6 hojas de cuadros más: en planners_hojas → id_planner: suena · portada: 1 · titulo: Notas · url: pagina-1-03.jpg · repetir: 6.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">hojas_actuales</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solo referencia (la web no la lee): cada hoja que hoy tiene cada planner, con su título y su archivo. portada 'todas' = la misma hoja en todas las portadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Imágenes</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">La planilla no guarda archivos: sube la imagen a Cloudinary (como las fotos del catálogo) y pega su URL. La web la achica sola.</t>
         </is>
@@ -374,6 +386,7 @@
     <col min="10" max="10" width="7" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -437,6 +450,11 @@
           <t xml:space="preserve">orientacion</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tipo</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
@@ -482,6 +500,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
@@ -527,6 +550,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M3" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
@@ -572,6 +600,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M4" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
@@ -617,6 +650,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M5" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
@@ -662,6 +700,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M6" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
@@ -707,6 +750,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M7" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
@@ -752,6 +800,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M8" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
@@ -797,6 +850,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M9" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
@@ -842,6 +900,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
@@ -887,6 +950,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M11" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
@@ -932,6 +1000,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M12" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
@@ -977,6 +1050,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M13" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
@@ -1022,6 +1100,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M14" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
@@ -1067,6 +1150,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M15" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
@@ -1112,6 +1200,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M16" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
@@ -1157,6 +1250,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
@@ -1202,6 +1300,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M18" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
@@ -1247,6 +1350,11 @@
           <t xml:space="preserve">apaisada</t>
         </is>
       </c>
+      <c r="M19" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
@@ -1292,6 +1400,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
@@ -1337,6 +1450,11 @@
           <t xml:space="preserve">vertical</t>
         </is>
       </c>
+      <c r="M21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
@@ -1382,6 +1500,11 @@
           <t xml:space="preserve">apaisada</t>
         </is>
       </c>
+      <c r="M22" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
@@ -1427,6 +1550,11 @@
           <t xml:space="preserve">apaisada</t>
         </is>
       </c>
+      <c r="M23" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tematica</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
@@ -1470,6 +1598,11 @@
       <c r="L24" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">apaisada</t>
+        </is>
+      </c>
+      <c r="M24" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">planner</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plantilla de planners: listas desplegables, formato de precio y filtros
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planners_heart_graphic.xlsx
+++ b/planners_heart_graphic.xlsx
@@ -13,6 +13,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -50,12 +53,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -472,7 +476,7 @@
           <t xml:space="preserve">Agenda Atrévete 2027</t>
         </is>
       </c>
-      <c r="D2" s="0">
+      <c r="D2" s="3">
         <v>14990</v>
       </c>
       <c r="F2" s="0" t="inlineStr">
@@ -480,12 +484,12 @@
           <t xml:space="preserve">B5</t>
         </is>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Agenda mes a mes con calendario, metas, control de gastos, ahorro y semana a la vista.</t>
         </is>
       </c>
-      <c r="H2" s="0" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño B5 de 17,6 × 25 cm, 100 hojas (200 páginas) anilladas</t>
         </is>
@@ -522,7 +526,7 @@
           <t xml:space="preserve">Mi Planner</t>
         </is>
       </c>
-      <c r="D3" s="0">
+      <c r="D3" s="3">
         <v>11990</v>
       </c>
       <c r="F3" s="0" t="inlineStr">
@@ -530,12 +534,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G3" s="0" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner con datos personales, calendario, semana a la vista y hábitos. Elige entre 3 diseños.</t>
         </is>
       </c>
-      <c r="H3" s="0" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -572,7 +576,7 @@
           <t xml:space="preserve">Planner Brilla</t>
         </is>
       </c>
-      <c r="D4" s="0">
+      <c r="D4" s="3">
         <v>11990</v>
       </c>
       <c r="F4" s="0" t="inlineStr">
@@ -580,12 +584,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G4" s="0" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner con calendarios 2026-2027, planificación mensual, gastos, hábitos y semana a la vista. Elige entre 2 portadas.</t>
         </is>
       </c>
-      <c r="H4" s="0" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -622,7 +626,7 @@
           <t xml:space="preserve">Planner Docente · Héroes</t>
         </is>
       </c>
-      <c r="D5" s="0">
+      <c r="D5" s="3">
         <v>9990</v>
       </c>
       <c r="F5" s="0" t="inlineStr">
@@ -630,12 +634,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G5" s="0" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner para profes: horario, evaluaciones y planificación semanal.</t>
         </is>
       </c>
-      <c r="H5" s="0" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· anillado</t>
         </is>
@@ -672,7 +676,7 @@
           <t xml:space="preserve">Planner Docente</t>
         </is>
       </c>
-      <c r="D6" s="0">
+      <c r="D6" s="3">
         <v>11990</v>
       </c>
       <c r="F6" s="0" t="inlineStr">
@@ -680,12 +684,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G6" s="0" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner para profes con calendarios 2026-2027, horario, evaluaciones y apoderados. Elige entre 2 diseños.</t>
         </is>
       </c>
-      <c r="H6" s="0" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -722,7 +726,7 @@
           <t xml:space="preserve">Planner Universitario</t>
         </is>
       </c>
-      <c r="D7" s="0">
+      <c r="D7" s="3">
         <v>11990</v>
       </c>
       <c r="F7" s="0" t="inlineStr">
@@ -730,12 +734,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G7" s="0" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner para la U con calendario 2027. Elige entre 6 portadas.</t>
         </is>
       </c>
-      <c r="H7" s="0" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -772,7 +776,7 @@
           <t xml:space="preserve">Planner Diario</t>
         </is>
       </c>
-      <c r="D8" s="0">
+      <c r="D8" s="3">
         <v>11990</v>
       </c>
       <c r="F8" s="0" t="inlineStr">
@@ -780,12 +784,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G8" s="0" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Un día por página para planificar con calma, con cumpleaños, hábitos y mes a mes. Elige entre 3 diseños.</t>
         </is>
       </c>
-      <c r="H8" s="0" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -822,7 +826,7 @@
           <t xml:space="preserve">Planner Diario · Anillado arriba</t>
         </is>
       </c>
-      <c r="D9" s="0">
+      <c r="D9" s="3">
         <v>7990</v>
       </c>
       <c r="F9" s="0" t="inlineStr">
@@ -830,12 +834,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G9" s="0" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Un día por página, con el anillado arriba. Elige entre 5 diseños.</t>
         </is>
       </c>
-      <c r="H9" s="0" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -872,7 +876,7 @@
           <t xml:space="preserve">Planner Semanal Diario</t>
         </is>
       </c>
-      <c r="D10" s="0">
+      <c r="D10" s="3">
         <v>11990</v>
       </c>
       <c r="F10" s="0" t="inlineStr">
@@ -880,12 +884,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G10" s="0" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planificación semanal y diaria con calendario. Elige entre 2 diseños.</t>
         </is>
       </c>
-      <c r="H10" s="0" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -922,7 +926,7 @@
           <t xml:space="preserve">Planner Sueña en Grande</t>
         </is>
       </c>
-      <c r="D11" s="0">
+      <c r="D11" s="3">
         <v>11990</v>
       </c>
       <c r="F11" s="0" t="inlineStr">
@@ -930,12 +934,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G11" s="0" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner tipo cuaderno con calendario y planificación mensual. Elige entre 2 diseños.</t>
         </is>
       </c>
-      <c r="H11" s="0" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -972,7 +976,7 @@
           <t xml:space="preserve">Diario de Gratitud</t>
         </is>
       </c>
-      <c r="D12" s="0">
+      <c r="D12" s="3">
         <v>11990</v>
       </c>
       <c r="F12" s="0" t="inlineStr">
@@ -980,12 +984,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G12" s="0" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Diario para agradecer cada día. Elige entre 2 portadas.</t>
         </is>
       </c>
-      <c r="H12" s="0" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -1022,7 +1026,7 @@
           <t xml:space="preserve">Planner Control de Gastos</t>
         </is>
       </c>
-      <c r="D13" s="0">
+      <c r="D13" s="3">
         <v>11990</v>
       </c>
       <c r="F13" s="0" t="inlineStr">
@@ -1030,12 +1034,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G13" s="0" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">“Planificarme es mi superpoder”: ingresos, gastos fijos, gastos hormiga, ahorros y balance del mes. Elige entre 2 portadas.</t>
         </is>
       </c>
-      <c r="H13" s="0" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 100 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -1072,7 +1076,7 @@
           <t xml:space="preserve">100 Citas Juntos</t>
         </is>
       </c>
-      <c r="D14" s="0">
+      <c r="D14" s="3">
         <v>9990</v>
       </c>
       <c r="F14" s="0" t="inlineStr">
@@ -1080,12 +1084,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G14" s="0" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Álbum de 100 citas para vivir en pareja: reglas, una página por cita con fotos, lugar, fecha y cómo se sintieron. Elige entre 3 portadas.</t>
         </is>
       </c>
-      <c r="H14" s="0" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -1122,7 +1126,7 @@
           <t xml:space="preserve">100 Citas con Amigas</t>
         </is>
       </c>
-      <c r="D15" s="0">
+      <c r="D15" s="3">
         <v>9990</v>
       </c>
       <c r="F15" s="0" t="inlineStr">
@@ -1130,12 +1134,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G15" s="0" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Álbum de citas para vivir con tus amigas: reglas, una página por cita con fotos y recuerdos. Elige entre 2 portadas.</t>
         </is>
       </c>
-      <c r="H15" s="0" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
         </is>
@@ -1172,7 +1176,7 @@
           <t xml:space="preserve">100 Citas con Mamá</t>
         </is>
       </c>
-      <c r="D16" s="0">
+      <c r="D16" s="3">
         <v>9990</v>
       </c>
       <c r="F16" s="0" t="inlineStr">
@@ -1180,12 +1184,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G16" s="0" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Álbum de 100 citas para compartir con mamá: carta, compromiso y una página por cita con foto.</t>
         </is>
       </c>
-      <c r="H16" s="0" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
         </is>
@@ -1222,7 +1226,7 @@
           <t xml:space="preserve">Carnet de Control Veterinario</t>
         </is>
       </c>
-      <c r="D17" s="0">
+      <c r="D17" s="3">
         <v>9990</v>
       </c>
       <c r="F17" s="0" t="inlineStr">
@@ -1230,12 +1234,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G17" s="0" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Agenda de control para tu gato o perro: datos, vacunas, desparasitación, controles y aseo. Elige entre 4 portadas.</t>
         </is>
       </c>
-      <c r="H17" s="0" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A5 (14,8 × 21 cm) · anillado</t>
         </is>
@@ -1272,7 +1276,7 @@
           <t xml:space="preserve">Agenda Mis Recetas</t>
         </is>
       </c>
-      <c r="D18" s="0">
+      <c r="D18" s="3">
         <v>7990</v>
       </c>
       <c r="F18" s="0" t="inlineStr">
@@ -1280,12 +1284,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G18" s="0" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Recetario para guardar tus recetas favoritas: ingredientes, tiempo, porciones y preparación. Elige entre 4 portadas.</t>
         </is>
       </c>
-      <c r="H18" s="0" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 (14,8 Ã 21 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -1322,7 +1326,7 @@
           <t xml:space="preserve">Planner Semanal</t>
         </is>
       </c>
-      <c r="D19" s="0">
+      <c r="D19" s="3">
         <v>7990</v>
       </c>
       <c r="F19" s="0" t="inlineStr">
@@ -1330,12 +1334,12 @@
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="G19" s="0" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Organiza tu semana a la vista. Elige entre 11 diseños: cada uno con su interior a juego.</t>
         </is>
       </c>
-      <c r="H19" s="0" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">TamaÃ±o A5 apaisado (21 Ã 14,8 cm) Â· 70 hojas de 106 g Â· anillado metÃ¡lico blanco</t>
         </is>
@@ -1372,7 +1376,7 @@
           <t xml:space="preserve">Mini Planner Diario</t>
         </is>
       </c>
-      <c r="D20" s="0">
+      <c r="D20" s="3">
         <v>5990</v>
       </c>
       <c r="F20" s="0" t="inlineStr">
@@ -1380,12 +1384,12 @@
           <t xml:space="preserve">A6</t>
         </is>
       </c>
-      <c r="G20" s="0" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner diario de bolsillo. Elige entre 5 portadas.</t>
         </is>
       </c>
-      <c r="H20" s="0" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A6 (10,5 × 14,8 cm) · anillado</t>
         </is>
@@ -1422,7 +1426,7 @@
           <t xml:space="preserve">Mini Agenda Líneas</t>
         </is>
       </c>
-      <c r="D21" s="0">
+      <c r="D21" s="3">
         <v>5990</v>
       </c>
       <c r="F21" s="0" t="inlineStr">
@@ -1430,12 +1434,12 @@
           <t xml:space="preserve">A6</t>
         </is>
       </c>
-      <c r="G21" s="0" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Agenda de bolsillo con hojas de líneas. Elige entre 4 portadas.</t>
         </is>
       </c>
-      <c r="H21" s="0" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A6 (10,5 × 14,8 cm) · anillado</t>
         </is>
@@ -1472,7 +1476,7 @@
           <t xml:space="preserve">Mini Planner Semanal</t>
         </is>
       </c>
-      <c r="D22" s="0">
+      <c r="D22" s="3">
         <v>5990</v>
       </c>
       <c r="F22" s="0" t="inlineStr">
@@ -1480,12 +1484,12 @@
           <t xml:space="preserve">A6</t>
         </is>
       </c>
-      <c r="G22" s="0" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Planner semanal de bolsillo con calendario y planificación mensual. Elige entre 5 portadas.</t>
         </is>
       </c>
-      <c r="H22" s="0" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A6 apaisado (14,8 × 10,5 cm) · anillado</t>
         </is>
@@ -1522,7 +1526,7 @@
           <t xml:space="preserve">Agenda Mis Pedidos</t>
         </is>
       </c>
-      <c r="D23" s="0">
+      <c r="D23" s="3">
         <v>5990</v>
       </c>
       <c r="F23" s="0" t="inlineStr">
@@ -1530,12 +1534,12 @@
           <t xml:space="preserve">A6</t>
         </is>
       </c>
-      <c r="G23" s="0" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Para emprendedoras: registra cada pedido con cliente, productos, pago y entrega. Elige entre 2 portadas.</t>
         </is>
       </c>
-      <c r="H23" s="0" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A6 apaisado (14,8 × 10,5 cm) · anillado</t>
         </is>
@@ -1572,7 +1576,7 @@
           <t xml:space="preserve">Mini Planner de Escritorio</t>
         </is>
       </c>
-      <c r="D24" s="0">
+      <c r="D24" s="3">
         <v>6990</v>
       </c>
       <c r="F24" s="0" t="inlineStr">
@@ -1580,12 +1584,12 @@
           <t xml:space="preserve">A6</t>
         </is>
       </c>
-      <c r="G24" s="0" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">“Pequeños planes, grandes logros”: pendientes del día y calendario. Elige entre 3 diseños.</t>
         </is>
       </c>
-      <c r="H24" s="0" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Tamaño A6 apaisado (14,8 × 10,5 cm) · anillado</t>
         </is>
@@ -1617,11 +1621,37 @@
           <t xml:space="preserve">precio personalización</t>
         </is>
       </c>
-      <c r="D25" s="0">
+      <c r="D25" s="3">
         <v>1000</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M25"/>
+  <dataValidations count="7">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="B2:B200">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Número no válido" error="Escribe un número entre 0 y 1000000" sqref="D2:D200">
+      <formula1>0</formula1>
+      <formula2>1000000</formula2>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Número no válido" error="Escribe un número entre 0 y 90" sqref="E2:E200">
+      <formula1>0</formula1>
+      <formula2>90</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="F2:F200">
+      <formula1>"B5,A5,A6"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="K2:K200">
+      <formula1>"costado,arriba"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="L2:L200">
+      <formula1>"vertical,apaisada"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="M2:M200">
+      <formula1>"planner,tematica"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -1675,6 +1705,16 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G2"/>
+  <dataValidations count="2">
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Número no válido" error="Escribe un número entre 1 y 99" sqref="B2:B200">
+      <formula1>1</formula1>
+      <formula2>99</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="G2:G200">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -1728,6 +1768,24 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G2"/>
+  <dataValidations count="4">
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Número no válido" error="Escribe un número entre 1 y 30" sqref="B2:B500">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Número no válido" error="Escribe un número entre 1 y 999" sqref="C2:C500">
+      <formula1>1</formula1>
+      <formula2>999</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elige una opción de la lista" sqref="F2:F500">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" allowBlank="1" showErrorMessage="1" errorTitle="Número no válido" error="Escribe un número entre 1 y 50" sqref="G2:G500">
+      <formula1>1</formula1>
+      <formula2>50</formula2>
+    </dataValidation>
+  </dataValidations>
 </worksheet>
 </file>
 
@@ -8601,5 +8659,6 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D332"/>
 </worksheet>
 </file>
</xml_diff>